<commit_message>
Prod Fixes On Edit Transfer, Payment-Module CHK
</commit_message>
<xml_diff>
--- a/TestFiles-prod-sanity/PaymentModule/ACH/[MLB][NB]PaymentModule-ACH.xlsx
+++ b/TestFiles-prod-sanity/PaymentModule/ACH/[MLB][NB]PaymentModule-ACH.xlsx
@@ -3,9 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25000" windowHeight="10000"/>
-  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
@@ -88,13 +85,13 @@
     <t>0987654321</t>
   </si>
   <si>
-    <t>232, E KING ST2 , ,, MALVERN, PA, 19355</t>
+    <t>232 E KING ST2 , ,, MALVERN, PA, 19355</t>
   </si>
   <si>
     <t>Integrity Health, LLC</t>
   </si>
   <si>
-    <t>AETNA-PAY-TEST-ACH-327</t>
+    <t>AETNA-PAY-TEST-ACH-033</t>
   </si>
   <si>
     <t>ROBERTS, PIPPIN</t>
@@ -116,10 +113,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -127,51 +121,16 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b/>
-      <i/>
-      <color theme="1"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <color rgb="FF000000"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -179,71 +138,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -272,28 +173,28 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285F4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="EA4335"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="FBBC04"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34A853"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="FF6D01"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46BDC6"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="0000FF"/>
@@ -406,20 +307,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -541,176 +438,187 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-  </sheetPr>
   <dimension ref="A1:U2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="9.140625"/>
-  <cols>
-    <col min="1" max="1" width="18.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.421875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.57421875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.57421875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="13.57421875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="29.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="19.421875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.8515625" style="3" customWidth="1"/>
-    <col min="10" max="10" width="13.57421875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.57421875" style="3" customWidth="1"/>
-    <col min="12" max="12" width="13.57421875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="13.57421875" style="4" customWidth="1"/>
-    <col min="15" max="15" width="13.57421875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="33.8515625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="13.57421875" style="3" customWidth="1"/>
-    <col min="19" max="20" width="13.57421875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="13.57421875" style="2" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" ht="19.5" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" spans="1:21" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="14">
+      <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="15">
-        <v>46388</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="I2" s="1">
+        <v>46023</v>
+      </c>
+      <c r="J2" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="15">
-        <v>46388</v>
-      </c>
-      <c r="L2" s="14">
+      <c r="K2" s="1">
+        <v>46023</v>
+      </c>
+      <c r="L2">
         <v>1</v>
       </c>
-      <c r="M2" s="16">
+      <c r="M2">
         <v>0</v>
       </c>
-      <c r="N2" s="16">
-        <v>78.9</v>
-      </c>
-      <c r="O2" s="14">
+      <c r="N2">
+        <v>54.9</v>
+      </c>
+      <c r="O2">
         <v>0</v>
       </c>
-      <c r="P2" s="14">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="5" t="s">
+      <c r="P2">
+        <v>48.31</v>
+      </c>
+      <c r="Q2" t="s">
         <v>29</v>
       </c>
-      <c r="R2" s="15">
-        <v>46388</v>
-      </c>
-      <c r="S2" s="5" t="s">
+      <c r="R2" s="1">
+        <v>46024</v>
+      </c>
+      <c r="S2" t="s">
         <v>30</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" t="s">
         <v>31</v>
       </c>
-      <c r="U2" s="14">
-        <v>789</v>
+      <c r="U2">
+        <v>549</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-  <headerFooter>
-    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
-    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>